<commit_message>
feat: enhance Dashboard and ValidationPanel with unknowns grid filter and subtype confusion matrix
</commit_message>
<xml_diff>
--- a/data/Subtypes.xlsx
+++ b/data/Subtypes.xlsx
@@ -2,16 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subtypes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Subtypes'!$A$1:$C$241</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -29,12 +26,14 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <family val="2"/>
+      <color rgb="FFffffff"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -47,32 +46,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E4057"/>
+        <fgColor rgb="FF2e4057"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0F4F8"/>
+        <fgColor rgb="FFf0f4f8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
+        <fgColor rgb="FFfff3cd"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8D5F5"/>
+        <fgColor rgb="FFe8d5f5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCE5FF"/>
+        <fgColor rgb="FFcce5ff"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D4EDDA"/>
+        <fgColor rgb="FFd4edda"/>
       </patternFill>
     </fill>
   </fills>
@@ -86,48 +85,52 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFcccccc"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFcccccc"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFcccccc"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFcccccc"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -206,10 +209,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -247,69 +250,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -333,54 +338,53 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="15000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
+                <a:tint val="94000"/>
                 <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
+              <a:shade val="9500"/>
               <a:satMod val="105000"/>
             </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -390,7 +394,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -399,7 +403,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -408,7 +412,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -416,10 +420,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -448,7 +452,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
+                <a:tint val="20000"/>
                 <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
@@ -461,13 +465,12 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
                 <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
+                <a:tint val="80000"/>
                 <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
@@ -487,18 +490,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="26.005" bestFit="1" customWidth="1" style="8" min="1" max="1"/>
+    <col width="20.005" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
+    <col width="30.005" bestFit="1" customWidth="1" style="8" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" hidden="1" ht="16.5" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Subtype</t>
@@ -515,7 +518,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" hidden="1" ht="16.5" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Developer</t>
@@ -528,11 +531,11 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" hidden="1" ht="16.5" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Education</t>
@@ -545,11 +548,11 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" hidden="1" ht="16.5" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Enterprise</t>
@@ -562,11 +565,11 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" hidden="1" ht="16.5" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Government</t>
@@ -579,11 +582,11 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" hidden="1" ht="16.5" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Nonprofit</t>
@@ -596,11 +599,11 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" hidden="1" ht="16.5" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Premium</t>
@@ -613,11 +616,11 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" hidden="1" ht="16.5" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Standard</t>
@@ -630,11 +633,11 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" hidden="1" ht="16.5" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Startup</t>
@@ -647,11 +650,11 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" hidden="1" ht="16.5" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Suspended</t>
@@ -664,11 +667,11 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" hidden="1" ht="16.5" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Trial</t>
@@ -681,11 +684,11 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" hidden="1" ht="16.5" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Unverified</t>
@@ -698,11 +701,11 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" hidden="1" ht="16.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Verified</t>
@@ -715,11 +718,11 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" hidden="1" ht="16.5" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Debug</t>
@@ -732,11 +735,11 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" hidden="1" ht="16.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Error</t>
@@ -749,11 +752,11 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" hidden="1" ht="16.5" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Info</t>
@@ -766,11 +769,11 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" hidden="1" ht="16.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Maintenance</t>
@@ -783,11 +786,11 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" hidden="1" ht="16.5" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Notification</t>
@@ -800,11 +803,11 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" hidden="1" ht="16.5" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Performance</t>
@@ -817,11 +820,11 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" hidden="1" ht="16.5" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Reminder</t>
@@ -834,11 +837,11 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" hidden="1" ht="16.5" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Security</t>
@@ -851,11 +854,11 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" hidden="1" ht="16.5" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Status</t>
@@ -868,11 +871,11 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" hidden="1" ht="16.5" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Success</t>
@@ -885,11 +888,11 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" hidden="1" ht="16.5" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Urgent</t>
@@ -902,11 +905,11 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" hidden="1" ht="16.5" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Warning</t>
@@ -919,11 +922,11 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" hidden="1" ht="16.5" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Attribution</t>
@@ -936,11 +939,11 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
+          <t>['France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" hidden="1" ht="16.5" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Click</t>
@@ -953,11 +956,11 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
+          <t>['France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" hidden="1" ht="16.5" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Cohort</t>
@@ -970,11 +973,11 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
+          <t>['France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" hidden="1" ht="16.5" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Conversion</t>
@@ -987,11 +990,11 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
+          <t>['France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" hidden="1" ht="16.5" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Engagement</t>
@@ -1004,11 +1007,11 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
+          <t>['France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" hidden="1" ht="16.5" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Funnel</t>
@@ -1021,11 +1024,11 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
+          <t>['France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" hidden="1" ht="16.5" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Pageview</t>
@@ -1038,11 +1041,11 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
+          <t>['France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" hidden="1" ht="16.5" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Retention</t>
@@ -1055,11 +1058,11 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
+          <t>['France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" hidden="1" ht="16.5" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Revenue</t>
@@ -1072,11 +1075,11 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
+          <t>['France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" hidden="1" ht="16.5" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Session</t>
@@ -1089,11 +1092,11 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
+          <t>['France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" hidden="1" ht="16.5" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Traffic</t>
@@ -1106,11 +1109,11 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
+          <t>['France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" hidden="1" ht="16.5" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
         <is>
           <t>User</t>
@@ -1123,11 +1126,11 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
+          <t>['France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" hidden="1" ht="16.5" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Alert</t>
@@ -1140,11 +1143,11 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" hidden="1" ht="16.5" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -1157,11 +1160,11 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" hidden="1" ht="16.5" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Chat</t>
@@ -1174,11 +1177,11 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" hidden="1" ht="16.5" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
         <is>
           <t>Email</t>
@@ -1191,11 +1194,11 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" hidden="1" ht="16.5" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
           <t>Forum</t>
@@ -1208,11 +1211,11 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" hidden="1" ht="16.5" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
         <is>
           <t>In App Message</t>
@@ -1225,11 +1228,11 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" hidden="1" ht="16.5" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Newsletter</t>
@@ -1242,11 +1245,11 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" hidden="1" ht="16.5" customHeight="1">
       <c r="A45" s="3" t="inlineStr">
         <is>
           <t>Phone Call</t>
@@ -1259,11 +1262,11 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" hidden="1" ht="16.5" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Push Notification</t>
@@ -1276,11 +1279,11 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" hidden="1" ht="16.5" customHeight="1">
       <c r="A47" s="3" t="inlineStr">
         <is>
           <t>SMS</t>
@@ -1293,11 +1296,11 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" hidden="1" ht="16.5" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Video Call</t>
@@ -1310,11 +1313,11 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" hidden="1" ht="16.5" customHeight="1">
       <c r="A49" s="3" t="inlineStr">
         <is>
           <t>WhatsApp</t>
@@ -1327,11 +1330,11 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" hidden="1" ht="16.5" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Billing</t>
@@ -1344,11 +1347,11 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" hidden="1" ht="16.5" customHeight="1">
       <c r="A51" s="3" t="inlineStr">
         <is>
           <t>Communication</t>
@@ -1361,11 +1364,11 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" hidden="1" ht="16.5" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Delivery</t>
@@ -1378,11 +1381,11 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" hidden="1" ht="16.5" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
         <is>
           <t>Discriminatory</t>
@@ -1395,11 +1398,11 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
           <t>Fraud</t>
@@ -1412,11 +1415,11 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" hidden="1" ht="16.5" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
         <is>
           <t>Misrepresentation</t>
@@ -1429,11 +1432,11 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" hidden="1" ht="16.5" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
           <t>Pricing</t>
@@ -1446,11 +1449,11 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" hidden="1" ht="16.5" customHeight="1">
       <c r="A57" s="3" t="inlineStr">
         <is>
           <t>Privacy</t>
@@ -1463,11 +1466,11 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" hidden="1" ht="16.5" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
           <t>Quality</t>
@@ -1480,11 +1483,11 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" hidden="1" ht="16.5" customHeight="1">
       <c r="A59" s="3" t="inlineStr">
         <is>
           <t>Safety</t>
@@ -1497,11 +1500,11 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" hidden="1" ht="16.5" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
           <t>Service</t>
@@ -1514,11 +1517,11 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" hidden="1" ht="16.5" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
         <is>
           <t>Support</t>
@@ -1531,11 +1534,11 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" hidden="1" ht="16.5" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
           <t>Archive</t>
@@ -1548,11 +1551,11 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" hidden="1" ht="16.5" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
         <is>
           <t>Audio</t>
@@ -1565,11 +1568,11 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" hidden="1" ht="16.5" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
           <t>Code</t>
@@ -1582,11 +1585,11 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" hidden="1" ht="16.5" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
         <is>
           <t>Comment</t>
@@ -1599,11 +1602,11 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" hidden="1" ht="16.5" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
           <t>Dataset</t>
@@ -1616,11 +1619,11 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" hidden="1" ht="16.5" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
           <t>Document</t>
@@ -1633,11 +1636,11 @@
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" hidden="1" ht="16.5" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
           <t>Image</t>
@@ -1650,11 +1653,11 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" hidden="1" ht="16.5" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
           <t>Presentation</t>
@@ -1667,11 +1670,11 @@
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" hidden="1" ht="16.5" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
           <t>Spreadsheet</t>
@@ -1684,11 +1687,11 @@
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" hidden="1" ht="16.5" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
         <is>
           <t>Text</t>
@@ -1701,11 +1704,11 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" hidden="1" ht="16.5" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
           <t>Video</t>
@@ -1718,11 +1721,11 @@
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" hidden="1" ht="16.5" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
         <is>
           <t>Webpage</t>
@@ -1735,11 +1738,11 @@
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" hidden="1" ht="16.5" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
           <t>Certificate</t>
@@ -1752,11 +1755,11 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" hidden="1" ht="16.5" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
         <is>
           <t>Contract</t>
@@ -1769,11 +1772,11 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" hidden="1" ht="16.5" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
           <t>Guide</t>
@@ -1786,11 +1789,11 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" hidden="1" ht="16.5" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
           <t>Invoice</t>
@@ -1803,11 +1806,11 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" hidden="1" ht="16.5" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
           <t>License</t>
@@ -1820,11 +1823,11 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" hidden="1" ht="16.5" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
         <is>
           <t>Manual</t>
@@ -1837,11 +1840,11 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" hidden="1" ht="16.5" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
           <t>Policy</t>
@@ -1854,11 +1857,11 @@
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" hidden="1" ht="16.5" customHeight="1">
       <c r="A81" s="3" t="inlineStr">
         <is>
           <t>Receipt</t>
@@ -1871,11 +1874,11 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" hidden="1" ht="16.5" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
           <t>Report</t>
@@ -1888,11 +1891,11 @@
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" hidden="1" ht="16.5" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
           <t>Shipping Label</t>
@@ -1905,11 +1908,11 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" hidden="1" ht="16.5" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
           <t>Terms</t>
@@ -1922,11 +1925,11 @@
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" hidden="1" ht="16.5" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
           <t>Warranty</t>
@@ -1939,11 +1942,11 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Spain, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
+          <t>['Spain', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" hidden="1" ht="16.5" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
           <t>Conference</t>
@@ -1956,11 +1959,11 @@
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" hidden="1" ht="16.5" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
           <t>Exclusive</t>
@@ -1973,11 +1976,11 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" hidden="1" ht="16.5" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
           <t>Hybrid</t>
@@ -1990,11 +1993,11 @@
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" hidden="1" ht="16.5" customHeight="1">
       <c r="A89" s="3" t="inlineStr">
         <is>
           <t>In Person</t>
@@ -2007,11 +2010,11 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" hidden="1" ht="16.5" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
           <t>Launch</t>
@@ -2024,11 +2027,11 @@
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" hidden="1" ht="16.5" customHeight="1">
       <c r="A91" s="3" t="inlineStr">
         <is>
           <t>Meetup</t>
@@ -2041,11 +2044,11 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" hidden="1" ht="16.5" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
           <t>Private</t>
@@ -2058,11 +2061,11 @@
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" hidden="1" ht="16.5" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
           <t>Public</t>
@@ -2075,11 +2078,11 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" hidden="1" ht="16.5" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
           <t>Sponsored</t>
@@ -2092,11 +2095,11 @@
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" hidden="1" ht="16.5" customHeight="1">
       <c r="A95" s="3" t="inlineStr">
         <is>
           <t>Virtual</t>
@@ -2109,11 +2112,11 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" hidden="1" ht="16.5" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
           <t>Webinar</t>
@@ -2126,11 +2129,11 @@
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" hidden="1" ht="16.5" customHeight="1">
       <c r="A97" s="3" t="inlineStr">
         <is>
           <t>Workshop</t>
@@ -2143,11 +2146,11 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" hidden="1" ht="16.5" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
           <t>Bug Report</t>
@@ -2160,11 +2163,11 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" hidden="1" ht="16.5" customHeight="1">
       <c r="A99" s="3" t="inlineStr">
         <is>
           <t>Comment</t>
@@ -2177,11 +2180,11 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" hidden="1" ht="16.5" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
           <t>Feature Request</t>
@@ -2194,11 +2197,11 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" hidden="1" ht="16.5" customHeight="1">
       <c r="A101" s="3" t="inlineStr">
         <is>
           <t>Improvement</t>
@@ -2211,11 +2214,11 @@
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" hidden="1" ht="16.5" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
@@ -2228,11 +2231,11 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" hidden="1" ht="16.5" customHeight="1">
       <c r="A103" s="3" t="inlineStr">
         <is>
           <t>Neutral</t>
@@ -2245,11 +2248,11 @@
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" hidden="1" ht="16.5" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
           <t>Positive</t>
@@ -2262,11 +2265,11 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" hidden="1" ht="16.5" customHeight="1">
       <c r="A105" s="3" t="inlineStr">
         <is>
           <t>Question</t>
@@ -2279,11 +2282,11 @@
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" hidden="1" ht="16.5" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
           <t>Rating</t>
@@ -2296,11 +2299,11 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" hidden="1" ht="16.5" customHeight="1">
       <c r="A107" s="3" t="inlineStr">
         <is>
           <t>Review</t>
@@ -2313,11 +2316,11 @@
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" hidden="1" ht="16.5" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
           <t>Suggestion</t>
@@ -2330,11 +2333,11 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" hidden="1" ht="16.5" customHeight="1">
       <c r="A109" s="3" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -2347,11 +2350,11 @@
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" hidden="1" ht="16.5" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
         <is>
           <t>Affiliate</t>
@@ -2364,11 +2367,11 @@
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" hidden="1" ht="16.5" customHeight="1">
       <c r="A111" s="3" t="inlineStr">
         <is>
           <t>Content</t>
@@ -2381,11 +2384,11 @@
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" hidden="1" ht="16.5" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
         <is>
           <t>Direct Mail</t>
@@ -2398,11 +2401,11 @@
       </c>
       <c r="C112" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" hidden="1" ht="16.5" customHeight="1">
       <c r="A113" s="3" t="inlineStr">
         <is>
           <t>Email Campaign</t>
@@ -2415,11 +2418,11 @@
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" hidden="1" ht="16.5" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
         <is>
           <t>Event</t>
@@ -2432,11 +2435,11 @@
       </c>
       <c r="C114" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" hidden="1" ht="16.5" customHeight="1">
       <c r="A115" s="3" t="inlineStr">
         <is>
           <t>Influencer</t>
@@ -2449,11 +2452,11 @@
       </c>
       <c r="C115" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" hidden="1" ht="16.5" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
         <is>
           <t>Paid Ads</t>
@@ -2466,11 +2469,11 @@
       </c>
       <c r="C116" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" hidden="1" ht="16.5" customHeight="1">
       <c r="A117" s="3" t="inlineStr">
         <is>
           <t>Partnership</t>
@@ -2483,11 +2486,11 @@
       </c>
       <c r="C117" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" hidden="1" ht="16.5" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
         <is>
           <t>PR</t>
@@ -2500,11 +2503,11 @@
       </c>
       <c r="C118" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" hidden="1" ht="16.5" customHeight="1">
       <c r="A119" s="3" t="inlineStr">
         <is>
           <t>Referral</t>
@@ -2517,11 +2520,11 @@
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" hidden="1" ht="16.5" customHeight="1">
       <c r="A120" s="2" t="inlineStr">
         <is>
           <t>Social Media</t>
@@ -2534,11 +2537,11 @@
       </c>
       <c r="C120" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" hidden="1" ht="16.5" customHeight="1">
       <c r="A121" s="3" t="inlineStr">
         <is>
           <t>Webinar</t>
@@ -2551,11 +2554,11 @@
       </c>
       <c r="C121" s="6" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
+          <t>['France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" hidden="1" ht="16.5" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
         <is>
           <t>Bank Transfer</t>
@@ -2568,11 +2571,11 @@
       </c>
       <c r="C122" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" hidden="1" ht="16.5" customHeight="1">
       <c r="A123" s="3" t="inlineStr">
         <is>
           <t>Cash</t>
@@ -2585,11 +2588,11 @@
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" hidden="1" ht="16.5" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
         <is>
           <t>Check</t>
@@ -2602,11 +2605,11 @@
       </c>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" hidden="1" ht="16.5" customHeight="1">
       <c r="A125" s="3" t="inlineStr">
         <is>
           <t>COD</t>
@@ -2619,11 +2622,11 @@
       </c>
       <c r="C125" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" hidden="1" ht="16.5" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
         <is>
           <t>Credit Card</t>
@@ -2636,11 +2639,11 @@
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" hidden="1" ht="16.5" customHeight="1">
       <c r="A127" s="3" t="inlineStr">
         <is>
           <t>Cryptocurrency</t>
@@ -2653,11 +2656,11 @@
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" hidden="1" ht="16.5" customHeight="1">
       <c r="A128" s="2" t="inlineStr">
         <is>
           <t>Debit Card</t>
@@ -2670,11 +2673,11 @@
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" hidden="1" ht="16.5" customHeight="1">
       <c r="A129" s="3" t="inlineStr">
         <is>
           <t>Digital Wallet</t>
@@ -2687,11 +2690,11 @@
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" hidden="1" ht="16.5" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
         <is>
           <t>Gift Card</t>
@@ -2704,11 +2707,11 @@
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" hidden="1" ht="16.5" customHeight="1">
       <c r="A131" s="3" t="inlineStr">
         <is>
           <t>Invoice</t>
@@ -2721,11 +2724,11 @@
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" hidden="1" ht="16.5" customHeight="1">
       <c r="A132" s="2" t="inlineStr">
         <is>
           <t>Prepaid</t>
@@ -2738,11 +2741,11 @@
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" hidden="1" ht="16.5" customHeight="1">
       <c r="A133" s="3" t="inlineStr">
         <is>
           <t>Subscription</t>
@@ -2755,11 +2758,11 @@
       </c>
       <c r="C133" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" hidden="1" ht="16.5" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
         <is>
           <t>Bundle</t>
@@ -2772,11 +2775,11 @@
       </c>
       <c r="C134" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" hidden="1" ht="16.5" customHeight="1">
       <c r="A135" s="3" t="inlineStr">
         <is>
           <t>Clearance</t>
@@ -2789,11 +2792,11 @@
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" hidden="1" ht="16.5" customHeight="1">
       <c r="A136" s="2" t="inlineStr">
         <is>
           <t>Custom</t>
@@ -2806,11 +2809,11 @@
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" hidden="1" ht="16.5" customHeight="1">
       <c r="A137" s="3" t="inlineStr">
         <is>
           <t>Digital</t>
@@ -2823,11 +2826,11 @@
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" hidden="1" ht="16.5" customHeight="1">
       <c r="A138" s="2" t="inlineStr">
         <is>
           <t>Exclusive</t>
@@ -2840,11 +2843,11 @@
       </c>
       <c r="C138" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" hidden="1" ht="16.5" customHeight="1">
       <c r="A139" s="3" t="inlineStr">
         <is>
           <t>Gift</t>
@@ -2857,11 +2860,11 @@
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" hidden="1" ht="16.5" customHeight="1">
       <c r="A140" s="2" t="inlineStr">
         <is>
           <t>Licensed</t>
@@ -2874,11 +2877,11 @@
       </c>
       <c r="C140" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" hidden="1" ht="16.5" customHeight="1">
       <c r="A141" s="3" t="inlineStr">
         <is>
           <t>Limited</t>
@@ -2891,11 +2894,11 @@
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" hidden="1" ht="16.5" customHeight="1">
       <c r="A142" s="2" t="inlineStr">
         <is>
           <t>Physical</t>
@@ -2908,11 +2911,11 @@
       </c>
       <c r="C142" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" hidden="1" ht="16.5" customHeight="1">
       <c r="A143" s="3" t="inlineStr">
         <is>
           <t>Refurbished</t>
@@ -2925,11 +2928,11 @@
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" hidden="1" ht="16.5" customHeight="1">
       <c r="A144" s="2" t="inlineStr">
         <is>
           <t>Rental</t>
@@ -2942,11 +2945,11 @@
       </c>
       <c r="C144" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" hidden="1" ht="16.5" customHeight="1">
       <c r="A145" s="3" t="inlineStr">
         <is>
           <t>Subscription</t>
@@ -2959,11 +2962,11 @@
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>Spain, France</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
+          <t>['Spain', 'France']</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" hidden="1" ht="16.5" customHeight="1">
       <c r="A146" s="2" t="inlineStr">
         <is>
           <t>Changed Mind</t>
@@ -2976,11 +2979,11 @@
       </c>
       <c r="C146" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" hidden="1" ht="16.5" customHeight="1">
       <c r="A147" s="3" t="inlineStr">
         <is>
           <t>Damaged in Transit</t>
@@ -2993,11 +2996,11 @@
       </c>
       <c r="C147" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" hidden="1" ht="16.5" customHeight="1">
       <c r="A148" s="2" t="inlineStr">
         <is>
           <t>Defective</t>
@@ -3010,11 +3013,11 @@
       </c>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" hidden="1" ht="16.5" customHeight="1">
       <c r="A149" s="3" t="inlineStr">
         <is>
           <t>Duplicate</t>
@@ -3027,11 +3030,11 @@
       </c>
       <c r="C149" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" hidden="1" ht="16.5" customHeight="1">
       <c r="A150" s="2" t="inlineStr">
         <is>
           <t>Expired</t>
@@ -3044,11 +3047,11 @@
       </c>
       <c r="C150" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" hidden="1" ht="16.5" customHeight="1">
       <c r="A151" s="3" t="inlineStr">
         <is>
           <t>Full</t>
@@ -3061,11 +3064,11 @@
       </c>
       <c r="C151" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" hidden="1" ht="16.5" customHeight="1">
       <c r="A152" s="2" t="inlineStr">
         <is>
           <t>Incompatible</t>
@@ -3078,11 +3081,11 @@
       </c>
       <c r="C152" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" hidden="1" ht="16.5" customHeight="1">
       <c r="A153" s="3" t="inlineStr">
         <is>
           <t>Not As Described</t>
@@ -3095,11 +3098,11 @@
       </c>
       <c r="C153" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" hidden="1" ht="16.5" customHeight="1">
       <c r="A154" s="2" t="inlineStr">
         <is>
           <t>Partial</t>
@@ -3112,11 +3115,11 @@
       </c>
       <c r="C154" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" hidden="1" ht="16.5" customHeight="1">
       <c r="A155" s="3" t="inlineStr">
         <is>
           <t>Recall</t>
@@ -3129,11 +3132,11 @@
       </c>
       <c r="C155" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" hidden="1" ht="16.5" customHeight="1">
       <c r="A156" s="2" t="inlineStr">
         <is>
           <t>Unwanted</t>
@@ -3146,11 +3149,11 @@
       </c>
       <c r="C156" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" hidden="1" ht="16.5" customHeight="1">
       <c r="A157" s="3" t="inlineStr">
         <is>
           <t>Wrong Item</t>
@@ -3163,11 +3166,11 @@
       </c>
       <c r="C157" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" hidden="1" ht="16.5" customHeight="1">
       <c r="A158" s="2" t="inlineStr">
         <is>
           <t>Access Control</t>
@@ -3180,11 +3183,11 @@
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" hidden="1" ht="16.5" customHeight="1">
       <c r="A159" s="3" t="inlineStr">
         <is>
           <t>Audit</t>
@@ -3197,11 +3200,11 @@
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" hidden="1" ht="16.5" customHeight="1">
       <c r="A160" s="2" t="inlineStr">
         <is>
           <t>Encryption</t>
@@ -3214,11 +3217,11 @@
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" hidden="1" ht="16.5" customHeight="1">
       <c r="A161" s="3" t="inlineStr">
         <is>
           <t>Firewall</t>
@@ -3231,11 +3234,11 @@
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" hidden="1" ht="16.5" customHeight="1">
       <c r="A162" s="2" t="inlineStr">
         <is>
           <t>Login</t>
@@ -3248,11 +3251,11 @@
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" hidden="1" ht="16.5" customHeight="1">
       <c r="A163" s="3" t="inlineStr">
         <is>
           <t>Password</t>
@@ -3265,11 +3268,11 @@
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" hidden="1" ht="16.5" customHeight="1">
       <c r="A164" s="2" t="inlineStr">
         <is>
           <t>Patch</t>
@@ -3282,11 +3285,11 @@
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" hidden="1" ht="16.5" customHeight="1">
       <c r="A165" s="3" t="inlineStr">
         <is>
           <t>Permission</t>
@@ -3299,11 +3302,11 @@
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" hidden="1" ht="16.5" customHeight="1">
       <c r="A166" s="2" t="inlineStr">
         <is>
           <t>Role</t>
@@ -3316,11 +3319,11 @@
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" hidden="1" ht="16.5" customHeight="1">
       <c r="A167" s="3" t="inlineStr">
         <is>
           <t>SSL</t>
@@ -3333,11 +3336,11 @@
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" hidden="1" ht="16.5" customHeight="1">
       <c r="A168" s="2" t="inlineStr">
         <is>
           <t>VPN</t>
@@ -3350,11 +3353,11 @@
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" hidden="1" ht="16.5" customHeight="1">
       <c r="A169" s="3" t="inlineStr">
         <is>
           <t>Vulnerability</t>
@@ -3367,11 +3370,11 @@
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" hidden="1" ht="16.5" customHeight="1">
       <c r="A170" s="2" t="inlineStr">
         <is>
           <t>Consultation</t>
@@ -3384,11 +3387,11 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" hidden="1" ht="16.5" customHeight="1">
       <c r="A171" s="3" t="inlineStr">
         <is>
           <t>Delivery</t>
@@ -3401,11 +3404,11 @@
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" hidden="1" ht="16.5" customHeight="1">
       <c r="A172" s="2" t="inlineStr">
         <is>
           <t>Express</t>
@@ -3418,11 +3421,11 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" hidden="1" ht="16.5" customHeight="1">
       <c r="A173" s="3" t="inlineStr">
         <is>
           <t>Installation</t>
@@ -3435,11 +3438,11 @@
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" hidden="1" ht="16.5" customHeight="1">
       <c r="A174" s="2" t="inlineStr">
         <is>
           <t>Maintenance</t>
@@ -3452,11 +3455,11 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" hidden="1" ht="16.5" customHeight="1">
       <c r="A175" s="3" t="inlineStr">
         <is>
           <t>Onsite</t>
@@ -3469,11 +3472,11 @@
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" hidden="1" ht="16.5" customHeight="1">
       <c r="A176" s="2" t="inlineStr">
         <is>
           <t>Phone</t>
@@ -3486,11 +3489,11 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" hidden="1" ht="16.5" customHeight="1">
       <c r="A177" s="3" t="inlineStr">
         <is>
           <t>Premium</t>
@@ -3503,11 +3506,11 @@
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" hidden="1" ht="16.5" customHeight="1">
       <c r="A178" s="2" t="inlineStr">
         <is>
           <t>Remote</t>
@@ -3520,11 +3523,11 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" hidden="1" ht="16.5" customHeight="1">
       <c r="A179" s="3" t="inlineStr">
         <is>
           <t>Standard</t>
@@ -3537,11 +3540,11 @@
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" hidden="1" ht="16.5" customHeight="1">
       <c r="A180" s="2" t="inlineStr">
         <is>
           <t>Support</t>
@@ -3554,11 +3557,11 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" hidden="1" ht="16.5" customHeight="1">
       <c r="A181" s="3" t="inlineStr">
         <is>
           <t>Training</t>
@@ -3571,11 +3574,11 @@
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" hidden="1" ht="16.5" customHeight="1">
       <c r="A182" s="2" t="inlineStr">
         <is>
           <t>Drop Off</t>
@@ -3588,11 +3591,11 @@
       </c>
       <c r="C182" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" hidden="1" ht="16.5" customHeight="1">
       <c r="A183" s="3" t="inlineStr">
         <is>
           <t>Express</t>
@@ -3605,11 +3608,11 @@
       </c>
       <c r="C183" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" hidden="1" ht="16.5" customHeight="1">
       <c r="A184" s="2" t="inlineStr">
         <is>
           <t>Fragile</t>
@@ -3622,11 +3625,11 @@
       </c>
       <c r="C184" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" hidden="1" ht="16.5" customHeight="1">
       <c r="A185" s="3" t="inlineStr">
         <is>
           <t>Hazmat</t>
@@ -3639,11 +3642,11 @@
       </c>
       <c r="C185" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" hidden="1" ht="16.5" customHeight="1">
       <c r="A186" s="2" t="inlineStr">
         <is>
           <t>Insured</t>
@@ -3656,11 +3659,11 @@
       </c>
       <c r="C186" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" hidden="1" ht="16.5" customHeight="1">
       <c r="A187" s="3" t="inlineStr">
         <is>
           <t>International</t>
@@ -3673,11 +3676,11 @@
       </c>
       <c r="C187" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" hidden="1" ht="16.5" customHeight="1">
       <c r="A188" s="2" t="inlineStr">
         <is>
           <t>Overnight</t>
@@ -3690,11 +3693,11 @@
       </c>
       <c r="C188" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" hidden="1" ht="16.5" customHeight="1">
       <c r="A189" s="3" t="inlineStr">
         <is>
           <t>Self Pickup</t>
@@ -3707,11 +3710,11 @@
       </c>
       <c r="C189" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" hidden="1" ht="16.5" customHeight="1">
       <c r="A190" s="2" t="inlineStr">
         <is>
           <t>Signature</t>
@@ -3724,11 +3727,11 @@
       </c>
       <c r="C190" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" hidden="1" ht="16.5" customHeight="1">
       <c r="A191" s="3" t="inlineStr">
         <is>
           <t>Standard</t>
@@ -3741,11 +3744,11 @@
       </c>
       <c r="C191" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" hidden="1" ht="16.5" customHeight="1">
       <c r="A192" s="2" t="inlineStr">
         <is>
           <t>Temperature Controlled</t>
@@ -3758,11 +3761,11 @@
       </c>
       <c r="C192" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" hidden="1" ht="16.5" customHeight="1">
       <c r="A193" s="3" t="inlineStr">
         <is>
           <t>White Glove</t>
@@ -3775,11 +3778,11 @@
       </c>
       <c r="C193" s="7" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
+          <t>['Spain']</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" hidden="1" ht="16.5" customHeight="1">
       <c r="A194" s="2" t="inlineStr">
         <is>
           <t>Callback</t>
@@ -3792,11 +3795,11 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" hidden="1" ht="16.5" customHeight="1">
       <c r="A195" s="3" t="inlineStr">
         <is>
           <t>Chat</t>
@@ -3809,11 +3812,11 @@
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" hidden="1" ht="16.5" customHeight="1">
       <c r="A196" s="2" t="inlineStr">
         <is>
           <t>Community</t>
@@ -3826,11 +3829,11 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" hidden="1" ht="16.5" customHeight="1">
       <c r="A197" s="3" t="inlineStr">
         <is>
           <t>Email</t>
@@ -3843,11 +3846,11 @@
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" hidden="1" ht="16.5" customHeight="1">
       <c r="A198" s="2" t="inlineStr">
         <is>
           <t>Escalation</t>
@@ -3860,11 +3863,11 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" hidden="1" ht="16.5" customHeight="1">
       <c r="A199" s="3" t="inlineStr">
         <is>
           <t>FAQ</t>
@@ -3877,11 +3880,11 @@
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" hidden="1" ht="16.5" customHeight="1">
       <c r="A200" s="2" t="inlineStr">
         <is>
           <t>In Person</t>
@@ -3894,11 +3897,11 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" hidden="1" ht="16.5" customHeight="1">
       <c r="A201" s="3" t="inlineStr">
         <is>
           <t>Knowledge Base</t>
@@ -3911,11 +3914,11 @@
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" hidden="1" ht="16.5" customHeight="1">
       <c r="A202" s="2" t="inlineStr">
         <is>
           <t>Phone</t>
@@ -3928,11 +3931,11 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" hidden="1" ht="16.5" customHeight="1">
       <c r="A203" s="3" t="inlineStr">
         <is>
           <t>Social Media</t>
@@ -3945,11 +3948,11 @@
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" hidden="1" ht="16.5" customHeight="1">
       <c r="A204" s="2" t="inlineStr">
         <is>
           <t>Ticket</t>
@@ -3962,11 +3965,11 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" hidden="1" ht="16.5" customHeight="1">
       <c r="A205" s="3" t="inlineStr">
         <is>
           <t>Video Tutorial</t>
@@ -3979,11 +3982,11 @@
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" hidden="1" ht="16.5" customHeight="1">
       <c r="A206" s="2" t="inlineStr">
         <is>
           <t>Authentication</t>
@@ -3996,11 +3999,11 @@
       </c>
       <c r="C206" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" hidden="1" ht="16.5" customHeight="1">
       <c r="A207" s="3" t="inlineStr">
         <is>
           <t>Backup</t>
@@ -4013,11 +4016,11 @@
       </c>
       <c r="C207" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" hidden="1" ht="16.5" customHeight="1">
       <c r="A208" s="2" t="inlineStr">
         <is>
           <t>Cache</t>
@@ -4030,11 +4033,11 @@
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" hidden="1" ht="16.5" customHeight="1">
       <c r="A209" s="3" t="inlineStr">
         <is>
           <t>Database</t>
@@ -4047,11 +4050,11 @@
       </c>
       <c r="C209" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" hidden="1" ht="16.5" customHeight="1">
       <c r="A210" s="2" t="inlineStr">
         <is>
           <t>Load Balancer</t>
@@ -4064,11 +4067,11 @@
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" hidden="1" ht="16.5" customHeight="1">
       <c r="A211" s="3" t="inlineStr">
         <is>
           <t>Logging</t>
@@ -4081,11 +4084,11 @@
       </c>
       <c r="C211" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" hidden="1" ht="16.5" customHeight="1">
       <c r="A212" s="2" t="inlineStr">
         <is>
           <t>Monitoring</t>
@@ -4098,11 +4101,11 @@
       </c>
       <c r="C212" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" hidden="1" ht="16.5" customHeight="1">
       <c r="A213" s="3" t="inlineStr">
         <is>
           <t>Network</t>
@@ -4115,11 +4118,11 @@
       </c>
       <c r="C213" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="214" hidden="1" ht="16.5" customHeight="1">
       <c r="A214" s="2" t="inlineStr">
         <is>
           <t>Queue</t>
@@ -4132,11 +4135,11 @@
       </c>
       <c r="C214" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" hidden="1" ht="16.5" customHeight="1">
       <c r="A215" s="3" t="inlineStr">
         <is>
           <t>Security</t>
@@ -4149,11 +4152,11 @@
       </c>
       <c r="C215" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" hidden="1" ht="16.5" customHeight="1">
       <c r="A216" s="2" t="inlineStr">
         <is>
           <t>Server</t>
@@ -4166,11 +4169,11 @@
       </c>
       <c r="C216" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" hidden="1" ht="16.5" customHeight="1">
       <c r="A217" s="3" t="inlineStr">
         <is>
           <t>Storage</t>
@@ -4183,11 +4186,11 @@
       </c>
       <c r="C217" s="4" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
+          <t>['Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" hidden="1" ht="16.5" customHeight="1">
       <c r="A218" s="2" t="inlineStr">
         <is>
           <t>Bulk</t>
@@ -4200,11 +4203,11 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" hidden="1" ht="16.5" customHeight="1">
       <c r="A219" s="3" t="inlineStr">
         <is>
           <t>Contract</t>
@@ -4217,11 +4220,11 @@
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" hidden="1" ht="16.5" customHeight="1">
       <c r="A220" s="2" t="inlineStr">
         <is>
           <t>Coupon</t>
@@ -4234,11 +4237,11 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="221" hidden="1" ht="16.5" customHeight="1">
       <c r="A221" s="3" t="inlineStr">
         <is>
           <t>Discount</t>
@@ -4251,11 +4254,11 @@
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" hidden="1" ht="16.5" customHeight="1">
       <c r="A222" s="2" t="inlineStr">
         <is>
           <t>Exchange</t>
@@ -4268,11 +4271,11 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" hidden="1" ht="16.5" customHeight="1">
       <c r="A223" s="3" t="inlineStr">
         <is>
           <t>Insurance</t>
@@ -4285,11 +4288,11 @@
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" hidden="1" ht="16.5" customHeight="1">
       <c r="A224" s="2" t="inlineStr">
         <is>
           <t>Promotion</t>
@@ -4302,11 +4305,11 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" hidden="1" ht="16.5" customHeight="1">
       <c r="A225" s="3" t="inlineStr">
         <is>
           <t>Purchase</t>
@@ -4319,11 +4322,11 @@
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="226">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" hidden="1" ht="16.5" customHeight="1">
       <c r="A226" s="2" t="inlineStr">
         <is>
           <t>Refund</t>
@@ -4336,11 +4339,11 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" hidden="1" ht="16.5" customHeight="1">
       <c r="A227" s="3" t="inlineStr">
         <is>
           <t>Subscription</t>
@@ -4353,11 +4356,11 @@
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" hidden="1" ht="16.5" customHeight="1">
       <c r="A228" s="2" t="inlineStr">
         <is>
           <t>Trial</t>
@@ -4370,11 +4373,11 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" hidden="1" ht="16.5" customHeight="1">
       <c r="A229" s="3" t="inlineStr">
         <is>
           <t>Warranty</t>
@@ -4387,11 +4390,11 @@
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="230">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" hidden="1" ht="16.5" customHeight="1">
       <c r="A230" s="2" t="inlineStr">
         <is>
           <t>Admin</t>
@@ -4404,11 +4407,11 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="231">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" hidden="1" ht="16.5" customHeight="1">
       <c r="A231" s="3" t="inlineStr">
         <is>
           <t>Corporate</t>
@@ -4421,11 +4424,11 @@
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="232">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" hidden="1" ht="16.5" customHeight="1">
       <c r="A232" s="2" t="inlineStr">
         <is>
           <t>Customer</t>
@@ -4438,11 +4441,11 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="233">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" hidden="1" ht="16.5" customHeight="1">
       <c r="A233" s="3" t="inlineStr">
         <is>
           <t>Free</t>
@@ -4455,11 +4458,11 @@
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="234">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" hidden="1" ht="16.5" customHeight="1">
       <c r="A234" s="2" t="inlineStr">
         <is>
           <t>Guest</t>
@@ -4472,11 +4475,11 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="235">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" hidden="1" ht="16.5" customHeight="1">
       <c r="A235" s="3" t="inlineStr">
         <is>
           <t>Inactive</t>
@@ -4489,11 +4492,11 @@
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="236">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" hidden="1" ht="16.5" customHeight="1">
       <c r="A236" s="2" t="inlineStr">
         <is>
           <t>Individual</t>
@@ -4506,11 +4509,11 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="237">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" hidden="1" ht="16.5" customHeight="1">
       <c r="A237" s="3" t="inlineStr">
         <is>
           <t>Influencer</t>
@@ -4523,11 +4526,11 @@
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="238">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" hidden="1" ht="16.5" customHeight="1">
       <c r="A238" s="2" t="inlineStr">
         <is>
           <t>Internal</t>
@@ -4540,11 +4543,11 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="239">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" hidden="1" ht="16.5" customHeight="1">
       <c r="A239" s="3" t="inlineStr">
         <is>
           <t>Partner</t>
@@ -4557,11 +4560,11 @@
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="240">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="240" hidden="1" ht="16.5" customHeight="1">
       <c r="A240" s="2" t="inlineStr">
         <is>
           <t>Premium</t>
@@ -4574,11 +4577,11 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
-        </is>
-      </c>
-    </row>
-    <row r="241" ht="16" customHeight="1">
+          <t>['Spain', 'France', 'Italy']</t>
+        </is>
+      </c>
+    </row>
+    <row r="241" hidden="1" ht="16.5" customHeight="1">
       <c r="A241" s="3" t="inlineStr">
         <is>
           <t>Vendor</t>
@@ -4591,12 +4594,11 @@
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Spain, France, Italy</t>
+          <t>['Spain', 'France', 'Italy']</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C241"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>